<commit_message>
updated the python scripts and created one for the api push methods so that it can be imported to the main file for execution
</commit_message>
<xml_diff>
--- a/Data/trane_news.xlsx
+++ b/Data/trane_news.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,191 +463,205 @@
           <t>source</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>attachmenturl</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Trane Technologies to Present at the Barclays Industrial Select Conference</t>
+          <t>Trane Technologies Completes Acquisition of Stellar Energy</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
           <t>SWORDS, Ireland--(BUSINESS WIRE)-- 
-Trane Technologies plc (NYSE: TT) a global climate innovator, today announced that company leadership will participate in a fireside chat at the Barclays Industrial Select Conference. They will speak at 9:15 a.m.</t>
+Trane Technologies (NYSE: TT), a global climate innovator, announced that it has completed the acquisition of Stellar Energy Americas, Inc. (“Stellar Energy”), a leading provider of turnkey data center cooling solutions. The acquisition was previously announced on December 2, 2025.</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46059</v>
+        <v>46071</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>SWORDS, Ireland--(BUSINESS WIRE)-- 
-Trane Technologies plc (NYSE: TT) a global climate innovator, today announced that company leadership will participate in a fireside chat at the Barclays Industrial Select Conference. They will speak at 9:15 a.m. ET on Tuesday, February 17, 2026. The live webcast will be accessible on the Trane Technologies website at www.tranetechnologies.com under the investor relations section. An archive of the webcast will be available for 30 days following the event.</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://investors.tranetechnologies.com/news-and-events/news-releases/news-release-details/2026/Trane-Technologies-to-Present-at-the-Barclays-Industrial-Select-Conference/default.aspx</t>
-        </is>
-      </c>
+Trane Technologies (NYSE: TT), a global climate innovator, announced that it has completed the acquisition of Stellar Energy Americas, Inc. (“Stellar Energy”), a leading provider of turnkey data center cooling solutions. The acquisition was previously announced on December 2, 2025. The acquisition strengthens Trane Technologies’ leadership in data center thermal management solutions, while accelerating growth, innovation and scale for Stellar Energy. Stellar Energy’s expertise in modular data center solutions combined with Trane Technologies’ operational excellence and global scale are well positioned to address the growing demand for pre-fabricated cooling systems and other critical equipment, which reduce supply chain constraints and enable rapid, scalable deployment. “The data center ecosystem is evolving rapidly, with growing demand for efficient, modular and scalable thermal management solutions, an area where Stellar Energy excels,” said Holly Paeper, President, Commercial HVAC Americas, Trane Technologies. “Their exceptional strength in modular thermal system design enhances our ability to lead as a trusted partner for this important sector as well as other complex commercial applications. We’re delighted to welcome the talented Stellar Energy team to Trane Technologies, and we look forward to building on their capabilities to deliver differentiated solutions that help customers achieve their growth, performance and sustainability goals.”</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>Trane Technologies</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>https://investors.tranetechnologies.com/news-and-events/news-releases/news-release-details/2026/Trane-Technologies-Completes-Acquisition-of-Stellar-Energy/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Trane Technologies to Present at the Citi Global Industrial Tech and Mobility Conference</t>
+          <t>Trane Technologies to Acquire LiquidStack to Accelerate End‑to‑End Data Center Thermal Management Solutions</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
           <t>SWORDS, Ireland--(BUSINESS WIRE)-- 
-Trane Technologies plc (NYSE: TT) a global climate innovator, today announced that company leadership will participate in a fireside chat at the Citi Global Industrial Tech Conference. They will speak at 10:30 a.m.</t>
+Trane Technologies (NYSE: TT), a global climate innovator, announced that it has entered into a definitive agreement to acquire LiquidStack, a global leader in liquid cooling technology for data centers, headquartered in Carrollton, Texas. LiquidStack solutions are engineered to meet the unprecedented demands of generative AI and hyperscale computing. Data centers and high‑performance compute organizations rely on LiquidStack for high-density liquid, direct-to-chip and immersion cooling solutions that improve efficiency, sustainability and performance.</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>46059</v>
+        <v>46063</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>SWORDS, Ireland--(BUSINESS WIRE)-- 
-Trane Technologies plc (NYSE: TT) a global climate innovator, today announced that company leadership will participate in a fireside chat at the Citi Global Industrial Tech Conference. They will speak at 10:30 a.m. ET on Wednesday, February 18, 2026. The live webcast will be accessible on the Trane Technologies website at www.tranetechnologies.com under the investor relations section. An archive of the webcast will be available for 30 days following the event.</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://investors.tranetechnologies.com/news-and-events/news-releases/news-release-details/2026/Trane-Technologies-to-Present-at-the-Citi-Global-Industrial-Tech-and-Mobility-Conference/default.aspx</t>
-        </is>
-      </c>
+Trane Technologies (NYSE: TT), a global climate innovator, announced that it has entered into a definitive agreement to acquire LiquidStack, a global leader in liquid cooling technology for data centers, headquartered in Carrollton, Texas. LiquidStack solutions are engineered to meet the unprecedented demands of generative AI and hyperscale computing. Data centers and high‑performance compute organizations rely on LiquidStack for high-density liquid, direct-to-chip and immersion cooling solutions that improve efficiency, sustainability and performance. Building on Trane Technologies’ minority investment in LiquidStack in 2023, this acquisition enhances Trane Technologies’ data center thermal management solutions, spanning chillers, heat rejection, controls, liquid distribution, and on‑chip cooling, and will scale LiquidStack’s pioneering technology globally. The acquisition includes LiquidStack’s highly skilled global team and manufacturing, engineering and research and development operations in Texas and Hong Kong. Upon closing, LiquidStack will operate globally within the Commercial HVAC business unit of the Trane Technologies Americas segment. “Rising chip‑level power and heat densities combined with increasingly variable workloads are redefining thermal management requirements inside modern data centers,” said Holly Paeper, President, Commercial HVAC Americas, Trane Technologies. “Customers need integrated cooling solutions that scale from the central plant to the chip and can adapt as performance demands continue to evolve. LiquidStack’s direct‑to‑chip and immersion cooling capabilities and talent, combined with Trane’s systems expertise and global footprint, strengthen our ability to deliver end‑to‑end, future‑ready thermal management across the entire data center ecosystem.” LiquidStack co-founder and CEO Joe Capes will join Trane Technologies in a leadership role and will continue to lead the LiquidStack business. “LiquidStack has been on a mission to innovate and deliver the most advanced, powerful and sustainable liquid cooling solutions,” said Joe Capes, CEO, LiquidStack. “Joining Trane Technologies enables us to accelerate that mission with the resources, scale and global reach needed to power next‑generation AI workloads in the most demanding compute environments. We are very excited to expand our impact and continue our growth as part of Trane Technologies.” The transaction is expected to close in early 2026, subject to closing conditions. Financial terms were not disclosed. This bolt-on acquisition follows Trane Technologies’ proven model of adding leading technologies that enhance its core businesses and scaling them to deliver strong returns over time. This follows the company’s recently-announced acquisition of Stellar Energy, which is expected to close in the first quarter of 2026.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>Trane Technologies</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>https://investors.tranetechnologies.com/news-and-events/news-releases/news-release-details/2026/Trane-Technologies-to-Acquire-LiquidStack-to-Accelerate-EndtoEnd-Data-Center-Thermal-Management-Solutions/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Trane Technologies Increases Dividend by 12%, Declares Quarterly Dividend</t>
+          <t>More from Trane Technologies</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SWORDS, Ireland--(BUSINESS WIRE)-- 
-Trane Technologies plc (NYSE:TT), a global climate innovator, announced the Board of Directors has approved a 12% increase to the company’s dividend, resulting in a quarterly dividend of $1.05 per ordinary share, or $4.20 per share annualized.</t>
+          <t>February 9, 2026 /3BL/ - Trane Technologies, a global climate innovator, is proud to announce that Reuben Trane will be inducted into the National Inventors Hall of Fame (NIHF) as a member of the 2026 class. This distinguished honor recognizes Trane’s legacy as a pioneering engineer whose vision and technological breakthroughs in heating, air conditioning and climate control transformed modern living, working and built environments. Reuben Trane co-founded The Trane Company in 1913 with his father, James, and sister, Stella in La Crosse, Wisconsin.</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>46057</v>
+        <v>46062.3125</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>SWORDS, Ireland--(BUSINESS WIRE)-- 
-Trane Technologies plc (NYSE:TT), a global climate innovator, announced the Board of Directors has approved a 12% increase to the company’s dividend, resulting in a quarterly dividend of $1.05 per ordinary share, or $4.20 per share annualized. The dividend is payable March 31, 2026, to shareholders of record on March 6, 2026. “Our purpose-driven strategy, disciplined execution and relentless investment in growth and innovation enables us to consistently deliver a leading growth profile, strong margins and powerful free cash flow,” said Dave Regnery, chair and CEO, Trane Technologies. “Since launching Trane Technologies in 2020, we have delivered free cash flow conversion of 106% of adjusted net earnings, enabling us to execute our balanced capital allocation strategy and nearly double the dividend. We are well positioned to deliver continued strong financial performance and differentiated shareholder returns over the long term.” Today’s announcement reflects the Company’s confidence in its ability to generate strong free cash flow in the future and pay a competitive and growing dividend over time. The Company has paid consecutive quarterly cash dividends on its common shares since 1919 and annual dividends since 1910.</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://investors.tranetechnologies.com/news-and-events/news-releases/news-release-details/2026/Trane-Technologies-Increases-Dividend-by-12-Declares-Quarterly-Dividend/default.aspx</t>
-        </is>
-      </c>
+          <t>February 9, 2026 /3BL/ - Trane Technologies, a global climate innovator, is proud to announce that Reuben Trane will be inducted into the National Inventors Hall of Fame (NIHF) as a member of the 2026 class. This distinguished honor recognizes Trane’s legacy as a pioneering engineer whose vision and technological breakthroughs in heating, air conditioning and climate control transformed modern living, working and built environments. Reuben Trane co-founded The Trane Company in 1913 with his father, James, and sister, Stella in La Crosse, Wisconsin. A mechanical engineer and prolific inventor, he is widely credited with advancing the HVAC industry through innovations such as the 1926 convector radiator, the coil which revolutionized building heating. Under his leadership, The Trane Company grew from a small family business into a global leader in sustainable climate solutions. His commitment to ingenuity, engineering excellence, and high‑quality design continues today and shapes the culture and mission of Trane Technologies. “Reuben Trane was ahead of his time—a visionary whose innovations have improved the comfort, health, and productivity of millions,” said Mauro Atalla, Senior Vice President and Chief Technology and Sustainability Officer, Trane Technologies. “His induction into the National Inventors Hall of Fame honors his pioneering contributions, which continue to influence who we are as a company. We proudly build on his legacy every day as we create bold solutions for a sustainable future.” Reuben Trane will be formally inducted into the National Inventors Hall of Fame on May 7, 2026. His great‑great‑grandson, Reuben Trane IV, a current Trane Technologies HVAC Systems Development Engineer, will accept the honor on his behalf. This recognition places Trane among an esteemed group of inventors whose contributions have advanced industries, strengthened global infrastructure, and significantly enhanced quality of life worldwide. Among this distinguished group is Frederick McKinley Jones, who was inducted into the National Inventors Hall of Fame in 2007. Jones invented the first portable air‑cooling unit for trucks in 1938 and co‑founded Thermo King two years later. Now part of Trane Technologies, Thermo King is the global leader in sustainable transport climate‑control solutions. ###</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>Trane Technologies</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>https://www.3blmedia.com/news/reuben-trane-named-2026-class-national-inventors-hall-fame</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ComfortSite Login</t>
+          <t>Trane Technologies to Present at the Barclays Industrial Select Conference</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Selecting a language changes the language and content on the Trane site. Trane ComfortSite is an extranet site designed to save you time. With your secure login, you can: This is the login for Trane® Connect™ and other Trane® commercial applications.</t>
+          <t>SWORDS, Ireland--(BUSINESS WIRE)-- 
+Trane Technologies plc (NYSE: TT) a global climate innovator, today announced that company leadership will participate in a fireside chat at the Barclays Industrial Select Conference. They will speak at 9:15 a.m.</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>46062.51324888301</v>
+        <v>46059</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Selecting a language changes the language and content on the Trane site. Trane ComfortSite is an extranet site designed to save you time. With your secure login, you can: This is the login for Trane® Connect™ and other Trane® commercial applications. Trane® Connect™ is our secure, cloud-based customer portal to access your building systems to remotely monitor and manage building systems, and conduct routine maintenance. Products Services Support Education &amp; Training Industries About North America Latin America Europe Middle East Asia Pacific Press Release Media Contact Trane Technologies Media Relations Trane by Trane Technologies Quick Facts DAVIDSON, N.C., Feb. 2, 2026 – Trane® – by Trane Technologies (NYSE: TT), a global climate innovator, today announced the launch of Trane Cloud, a digital hub designed to transform how building operators, facility teams, and energy managers interact with their buildings. Trane Cloud brings together analytics, applications and services into one secure, seamless digital experience, empowering teams to operate buildings more efficiently, reliably and sustainably. For years, building professionals have navigated a complex web of systems, with valuable data often trapped in proprietary interfaces or fragmented dashboards. Trane Cloud addresses this challenge by creating a single, intelligent data foundation that provides portfolio- and site-level visibility, delivering actionable insights for energy optimization and prioritized recommendations to streamline operations and enhance decision-making. “In today’s increasingly digital world, building operators are flooded with data from their buildings and need a way to make sense of it all,” said Riaz Raihan, Senior Vice President and Chief Digital Officer of Trane Technologies. “Trane Cloud is our answer. It serves as the entry point for the digital experience, revolutionizing building operations by bringing everything together in one place to optimize performance. Trane Cloud is the foundation for a smarter, more efficient building, helping our customers meet their goals for sustainability, efficiency, reliability and comfort.” Trane Cloud delivers a powerful suite of Trane applications and digital services to help building teams manage and prioritize their work more effectively. Key benefits of Trane Cloud include: Trane Cloud is designed for a wide range of customers, including facility teams focused on efficient operations; building teams focused on long-term performance; energy managers aiming to reduce carbon emissions; and organizations of all sizes seeking consistent, data-driven oversight across their portfolios. By providing a secure, scalable, and intuitive platform, Trane is empowering customers to unlock the full potential of their buildings.</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://www.trane.com/commercial/north-america/us/en/about-us/newsroom/press-releases/introducing-trane-cloud.html</t>
-        </is>
-      </c>
+          <t>SWORDS, Ireland--(BUSINESS WIRE)-- 
+Trane Technologies plc (NYSE: TT) a global climate innovator, today announced that company leadership will participate in a fireside chat at the Barclays Industrial Select Conference. They will speak at 9:15 a.m. ET on Tuesday, February 17, 2026. The live webcast will be accessible on the Trane Technologies website at www.tranetechnologies.com under the investor relations section. An archive of the webcast will be available for 30 days following the event.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>Trane Technologies</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>https://investors.tranetechnologies.com/news-and-events/news-releases/news-release-details/2026/Trane-Technologies-to-Present-at-the-Barclays-Industrial-Select-Conference/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ComfortSite Login</t>
+          <t>Trane Technologies to Present at the Citi Global Industrial Tech and Mobility Conference</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Selecting a language changes the language and content on the Trane site. Trane ComfortSite is an extranet site designed to save you time. With your secure login, you can: This is the login for Trane® Connect™ and other Trane® commercial applications.</t>
+          <t>SWORDS, Ireland--(BUSINESS WIRE)-- 
+Trane Technologies plc (NYSE: TT) a global climate innovator, today announced that company leadership will participate in a fireside chat at the Citi Global Industrial Tech Conference. They will speak at 10:30 a.m.</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>46062.51325268688</v>
+        <v>46059</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Selecting a language changes the language and content on the Trane site. Trane ComfortSite is an extranet site designed to save you time. With your secure login, you can: This is the login for Trane® Connect™ and other Trane® commercial applications. Trane® Connect™ is our secure, cloud-based customer portal to access your building systems to remotely monitor and manage building systems, and conduct routine maintenance. Products Services Support Education &amp; Training Industries About North America Latin America Europe Middle East Asia Pacific Press Release Garrett Motion’s breakthrough oil-free centrifugal compressor technology exclusively available through Trane portfolio for commercial applications. Media Contact Trane Technologies Media Relations Trane by Trane Technologies Quick Facts DAVIDSON, N.C., PLYMOUTH, MI, and ROLLE, Switzerland, Feb. 2, 2026 – Trane® – by Trane Technologies (NYSE: TT), a global climate innovator, and Garrett Motion (Nasdaq: GTX), a global leader in differentiated turbocharging and electrification technologies, today announced a strategic collaboration to accelerate next generation, oil-free centrifugal compressor technology for commercial heating, ventilation and air conditioning (HVAC) applications. The collaboration brings together Trane’s industry-leading Commercial HVAC system expertise and performance with Garrett’s breakthrough oil-free high-speed centrifugal compressor technology, which has already demonstrated clear performance benefits including major energy efficiency gains in Trane’s testing. Together, Trane and Garrett will launch the next generation of high efficiency HVAC systems and accelerate the adoption of ultra-low global warming potential refrigerants. The companies will jointly develop and integrate advanced compressor solutions across a broad portfolio of Trane systems, including unitary rooftop units, modular chillers, and large capacity chillers for a variety of applications. Field testing and production of the jointly developed technology are scheduled to begin in 2026, marking a major milestone in the companies’ shared focus on innovation, energy efficiency and lower environmental impact. “This collaboration advances our commitment to lead the industry with high-performing, energy efficient solutions that support our customers’ decarbonization goals,” said Mauro Atalla, Chief Technology and Sustainability Officer, Trane Technologies. “Garrett Motion brings deep expertise and a shared commitment to quality with their oil-free centrifugal compressor technology. Together, we are accelerating innovation that will shape the next era of sustainable HVAC systems.” The collaboration establishes a framework for shared engineering, design and field testing activities across global markets. It also includes joint exploration of future applications, including high-speed centrifugal technologies for smaller capacity HVAC systems, distributed cooling and other emerging cooling needs. “Garrett is proud to partner with Trane Technologies, one of the most respected names in the HVAC industry, as we expand the use of our unique oil-free high-speed compressor technology in the industrial space,” said Olivier Rabiller, President and CEO of Garrett Motion. “Combining this technology proven in several automotive applications with Trane’s system-level leadership enables customers to benefit from a better, more energy-efficient and cost-effective HVAC system while advancing their sustainability goals.” The collaboration reinforces both organizations’ commitment to industry-leading performance, reliability and customer value.</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://www.trane.com/commercial/north-america/us/en/about-us/newsroom/press-releases/garrett-motion-collab.html</t>
-        </is>
-      </c>
+          <t>SWORDS, Ireland--(BUSINESS WIRE)-- 
+Trane Technologies plc (NYSE: TT) a global climate innovator, today announced that company leadership will participate in a fireside chat at the Citi Global Industrial Tech Conference. They will speak at 10:30 a.m. ET on Wednesday, February 18, 2026. The live webcast will be accessible on the Trane Technologies website at www.tranetechnologies.com under the investor relations section. An archive of the webcast will be available for 30 days following the event.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>Trane Technologies</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>https://investors.tranetechnologies.com/news-and-events/news-releases/news-release-details/2026/Trane-Technologies-to-Present-at-the-Citi-Global-Industrial-Tech-and-Mobility-Conference/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Trane Technologies Reports Strong Fourth-Quarter and Full-Year 2025 Results; Robust Bookings and Backlog Provide Strong Visibility Entering 2026</t>
+          <t>Trane Technologies Increases Dividend by 12%, Declares Quarterly Dividend</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Highlights (fourth-quarter 2025 versus fourth-quarter 2024, unless otherwise noted): Highlights (full-year 2025 versus full-year 2024, unless otherwise noted): *This news release contains non-GAAP financial measures. Definitions of the non-GAAP financial measures can be found in the footnotes of this news release. See attached tables for additional details and reconciliations.</t>
+          <t>SWORDS, Ireland--(BUSINESS WIRE)-- 
+Trane Technologies plc (NYSE:TT), a global climate innovator, announced the Board of Directors has approved a 12% increase to the company’s dividend, resulting in a quarterly dividend of $1.05 per ordinary share, or $4.20 per share annualized.</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>46051</v>
+        <v>46057</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Highlights (fourth-quarter 2025 versus fourth-quarter 2024, unless otherwise noted): Highlights (full-year 2025 versus full-year 2024, unless otherwise noted): *This news release contains non-GAAP financial measures. Definitions of the non-GAAP financial measures can be found in the footnotes of this news release. See attached tables for additional details and reconciliations. SWORDS, Ireland--(BUSINESS WIRE)-- 
-Trane Technologies plc (NYSE:TT), a global climate innovator, today reported diluted earnings per share (EPS) from continuing operations of $2.74 for the fourth quarter of 2025. Adjusted continuing EPS was $2.86, up 10 percent. Fourth-Quarter 2025 Results Financial Comparisons - Fourth-Quarter Continuing Operations $, millions except EPS Q4 2025 Q4 2024 Y-O-Y Change Organic Y-O-Y Change Bookings $5,760 $4,659 24% 22% Net Revenues $5,145 $4,874 6% 4% GAAP Operating Income $819 $808 1%  GAAP Operating Margin 15.9% 16.6% (70) bps Adjusted Operating Income* $837 $794 5% Adjusted Operating Margin* 16.3% 16.3% 0 bps Adjusted EBITDA* $923 $894 3% Adjusted EBITDA Margin* 17.9% 18.3% (40) bps GAAP Continuing EPS $2.74 $2.67 3% Adjusted Continuing EPS $2.86 $2.61 10% Pre-tax Non-GAAP Adjustments, net** $34.9 ($13.2) $48.1 **For details see tables 2 and 3 of the news release. “Thanks to our purpose-driven strategy, talented team and disciplined execution, 2025 was another strong year for our company,” said Dave Regnery, chair and CEO. “We achieved strong revenue growth, adjusted earnings per share growth and free cash flow conversion, despite challenging markets in residential and transport refrigeration. "We continue to see tremendous strength and rapidly growing pipelines in our commercial HVAC businesses, led by the Americas, where fourth quarter applied bookings were up more than 120%. We ended the year with record enterprise backlog of $7.8 billion, providing strong visibility to future market outgrowth. “Since launching Trane Technologies in 2020, we’ve built a powerful long-term track record – including compound annual revenue growth of 11%, EBITDA margin expansion of 470 basis points, compound annual adjusted earnings per share growth of 24%, and free cash flow conversion of 106%. With significant opportunities ahead, record backlog levels and strong customer demand, we remain confident in delivering differentiated results into the future.” Highlights from the Fourth Quarter of 2025 (all comparisons against fourth-quarter 2024 unless otherwise noted): Fourth-Quarter Business Review (all comparisons against fourth-quarter 2024 unless otherwise noted) Americas Segment: innovates for customers in the North America and Latin America regions. The Americas segment encompasses commercial heating, cooling and ventilation systems, building controls and solutions, energy services and solutions, residential heating and cooling; and transport refrigeration systems and solutions. $, millions Q4 2025 Q4 2024 Y-O-Y Change Organic Y-O-Y Change Bookings $4,651.3 $3,676.5 27% 26% Net Revenues $4,012.6 $3,802.5 6% 5% GAAP Operating Income $686.7 $685.0 0%  GAAP Operating Margin 17.1% 18.0% (90) bps Adjusted Operating Income $691.8 $669.3 3% Adjusted Operating Margin 17.2% 17.6% (40) bps Adjusted EBITDA $757.2 $741.4 2% Adjusted EBITDA Margin 18.9% 19.5% (60) bps Europe, Middle East and Africa (EMEA) Segment: innovates for customers in the Europe, Middle East and Africa region. The EMEA segment encompasses heating, cooling and ventilation systems and services, energy services and solutions, and transport refrigeration systems and solutions. $, millions Q4 2025 Q4 2024 Y-O-Y Change Organic Y-O-Y Change Bookings $731.8 $614.8 19% 9% Net Revenues $771.0 $690.3 12% 2% GAAP Operating Income $122.0 $119.8 2%  GAAP Operating Margin 15.8% 17.4% (160) bps Adjusted Operating Income $124.6 $119.1 5% Adjusted Operating Margin 16.2% 17.3% (110) bps Adjusted EBITDA $133.7 $130.4 3% Adjusted EBITDA Margin 17.3% 18.9% (160) bps Asia Pacific Segment: innovates for customers throughout the Asia Pacific region. The Asia Pacific segment encompasses heating, cooling and ventilation systems, services and solutions for commercial buildings and transport refrigeration systems and solutions. $, millions Q4 2025 Q4 2024 Y-O-Y Change Organic Y-O-Y Change Bookings $376.8 $367.8 2% 1% Net Revenues $360.9 $381.2 (5)% (6)% GAAP Operating Income $92.7 $94.3 (2)%  GAAP Operating Margin 25.7% 24.7% 100 bps Adjusted Operating Income $92.7 $96.1 (4)% Adjusted Operating Margin 25.7% 25.2% 50 bps Adjusted EBITDA $95.0 $100.9 (6)% Adjusted EBITDA Margin 26.3% 26.5% (20) bps Full-Year 2025 Results (all comparisons against full-year 2024 unless otherwise noted) Financial Comparisons - Full-year Continuing Operations $, millions except EPS 2025 2024 Y-O-Y Change Organic Y-O-Y Bookings $22,648 $20,286 12% 11% Net Revenues $21,322 $19,838 7% 6% GAAP Operating Income $3,967 $3,500 13%  GAAP Operating Margin 18.6% 17.6% 100 bps Adjusted Operating Income $3,945 $3,487 13% Adjusted Operating Margin 18.5% 17.6% 90 bps Adjusted EBITDA $4,276 $3,846 11% Adjusted EBITDA Margin 20.1% 19.4% 70 bps GAAP Continuing EPS $13.14 $11.35 16% Adjusted Continuing EPS $13.06 $11.22 16% Balance Sheet and Cash Flow $, millions 2025 2024 Y-O-Y Change Cash From Continuing Operating Activities Y-T-D $3,220 $3,178 $42 Free Cash Flow Y-T-D* $2,887 $2,789 $98 Working Capital/Revenue* 2.4% 0.8% 160 bps increase Cash Balance 31 December $1,763 $1,590 $173 Debt Balance 31 December $4,615 $4,770 ($155) Full-Year 2026 Guidance This news release includes “forward-looking" statements within the meaning of securities laws, which are statements that are not historical facts, including statements that relate to our future financial performance and targets, including revenue, EPS, and earnings; our business operations; demand for our products and services, including bookings and backlog; capital deployment, including the amount and timing of our dividends, our share repurchase program, anticipated capital commitments for M&amp;A activity, and our capital allocation strategy; our available liquidity; our anticipated revenue growth, and the performance of the markets in which we operate. These forward-looking statements are based on our current expectations and are subject to risks and uncertainties, which may cause actual results to differ materially from our current expectations. Such factors include, but are not limited to, global economic conditions, including recessions and economic downturns, inflation, volatility in interest rates and foreign exchange; trade protection measures such as import or export restrictions, tariffs, quotas; or modifications trade agreements; changing energy prices; worldwide geopolitical conflict; financial institution disruptions; climate change and our sustainability strategies and goals; future health care emergencies on our business, our suppliers and our customers; commodity shortages; price increases; government regulation; restructurings activity and cost savings associated with such activity; secular trends toward decarbonization, energy efficiency and internal air quality, the outcome of any litigation, including the risks and uncertainties associated with the Chapter 11 proceedings for our deconsolidated subsidiaries Aldrich Pump LLC and Murray Boiler LLC; cybersecurity risks; and tax audits and tax law changes and interpretations. Additional factors that could cause such differences can be found in our Form 10-K for the year ended December 31, 2025, as well as our subsequent reports on Form 10-Q and other SEC filings. New risks and uncertainties arise from time to time, and it is impossible for us to predict these events and how they may affect the Company. We assume no obligation to update these forward-looking statements. This news release also includes non-GAAP financial information, which should be considered supplemental to, not a substitute for, or superior to, the financial measure calculated in accordance with GAAP. The definitions of our non-GAAP financial information and reconciliation to GAAP are attached to this news release. All amounts reported within the earnings release above related to net earnings (loss), earnings (loss) from continuing operations, earnings (loss) from discontinued operations, adjusted EBITDA and per share amounts are attributed to Trane Technologies' ordinary shareholders. Trane Technologies (NYSE:TT) is a global climate innovator. Through our strategic brands Trane® and Thermo King®, and our portfolio of environmentally responsible products and services, we bring efficient and sustainable climate solutions to buildings, homes and transportation. For more information, visit tranetechnologies.com. # # # 1/29/26 (See Accompanying Tables) *Q4 Year-to-Date Non-GAAP measures definitions Adjusted operating income in 2025 is defined as GAAP operating income adjusted for restructuring costs, merger and acquisition transaction costs, and a non-cash adjustment for contingent consideration. Adjusted operating income in 2024 is defined as GAAP operating income adjusted for restructuring costs, legacy legal liability, merger and acquisition transaction costs, and a non-cash adjustment for contingent consideration. Please refer to the reconciliation of GAAP to non-GAAP measures on tables 2, 3, 4 and 5 of the news release. Adjusted operating margin is defined as the ratio of adjusted operating income divided by net revenues. Adjusted net earnings from continuing operations attributable to Trane Technologies plc (Adjusted net earnings) in 2025 is defined as GAAP earnings from continuing operations attributable to Trane Technologies plc adjusted for net of tax impacts of restructuring costs, merger and acquisition transaction costs, a non-cash adjustment for contingent consideration, and a non-cash settlement charge related to the transfer of a pension liability to an insurance company. Adjusted net earnings in 2024 is defined as GAAP earnings from continuing operations attributable to Trane Technologies plc adjusted for net of tax impacts of restructuring costs, legacy legal liability, merger and acquisition transaction costs, a non-cash adjustment for contingent consideration, and a U.S. discrete tax benefit. Please refer to the reconciliation of GAAP to non-GAAP measures on tables 2 and 3 of the news release. Adjusted continuing EPS in 2025 is defined as GAAP continuing EPS adjusted for net of tax impacts of restructuring costs, merger and acquisition transaction costs, a non-cash adjustment for contingent consideration, and a non-cash settlement charge related to the transfer of a pension liability to an insurance company. Adjusted continuing EPS in 2024 is defined as GAAP continuing EPS adjusted for net of tax impacts of restructuring costs, legacy legal liability, merger and acquisition transaction costs, a non-cash adjustment for contingent consideration, and a U.S. discrete tax benefit. Please refer to the reconciliation of GAAP to non-GAAP measures on tables 2 and 3 of the news release. Adjusted EBITDA in 2025 is defined as adjusted operating income excluding depreciation and amortization expense and including other income / (expense), net, adjusted for a non-cash settlement charge related to the transfer of a pension liability to an insurance company. Adjusted EBITDA in 2024 is defined as adjusted operating income excluding depreciation and amortization expense and including other income / (expense), net. Other income / (expense), net mainly comprises interest income, foreign currency exchange gains and losses and certain components of pension and postretirement benefit costs. Please refer to the reconciliation of GAAP to non-GAAP measures on tables 4, 5, 6 and 7 of the news release. Adjusted EBITDA margin is defined as the ratio of adjusted EBITDA divided by net revenues. Adjusted effective tax rate for 2025 is defined as the ratio of income tax expense adjusted for the net tax effect of adjustments for restructuring costs, merger and acquisition transaction costs, and a non-cash settlement charge related to the transfer of a pension liability to an insurance company divided by adjusted net earnings. Adjusted effective tax rate for 2024 is defined as the ratio of income tax expense adjusted for the net tax effect of adjustments restructuring costs, legacy legal liability, and merger and acquisition transaction costs, divided by adjusted net earnings. This measure allows for a direct comparison of the effective tax rate between periods. Free cash flow in 2025 is defined as net cash provided by (used in) continuing operating activities adjusted for capital expenditures, cash payments for restructuring costs, legacy legal liability, merger and acquisition transaction costs and proceeds from sale of corporate asset. Free cash flow in 2024 is defined as net cash provided by (used in) continuing operating activities adjusted for capital expenditures, cash payments for restructuring costs, legacy legal liability, and merger and acquisition transaction costs less an adjustment for a special three-year Outperformance Incentive Program. Please refer to the free cash flow reconciliation on table 10 of the news release. Operating leverage is defined as the ratio of the change in adjusted operating income for the current period (e.g. Q4 2025) less the prior period (e.g. Q4 2024), divided by the change in net revenues for the current period less the prior period. Organic revenue is defined as GAAP net revenues adjusted for the impact of currency and acquisitions. Organic bookings is defined as reported orders in the current period adjusted for the impact of currency and acquisitions. Working capital measures a firm’s operating liquidity position and its overall effectiveness in managing the enterprise's current accounts. The Company reports its financial results in accordance with generally accepted accounting principles in the United States (GAAP). The following schedules provide non-GAAP financial information and a quantitative reconciliation of the difference between the non-GAAP financial measures and the financial measures calculated and reported in accordance with GAAP. The non-GAAP financial measures should be considered supplemental to, not a substitute for or superior to, financial measures calculated in accordance with GAAP. They have limitations in that they do not reflect all of the costs associated with the operations of our businesses as determined in accordance with GAAP. In addition, these measures may not be comparable to non-GAAP financial measures reported by other companies. We believe the non-GAAP financial information provides important supplemental information to both management and investors regarding financial and business trends used in assessing our financial condition and results of operations. Non-GAAP financial measures assist investors with analyzing our business results as well as with predicting future performance. In addition, these non-GAAP financial measures are also reviewed by management in order to evaluate the financial performance of each segment. Presentation of these non-GAAP financial measures helps investors and management to assess the operating performance of the Company. As a result, one should not consider these measures in isolation or as a substitute for our results reported under GAAP. We compensate for these limitations by analyzing results on a GAAP basis as well as a non-GAAP basis, prominently disclosing GAAP results and providing reconciliations from GAAP results to non-GAAP results. Table 1 TRANE TECHNOLOGIES PLC Condensed Consolidated Income Statement (In millions, except per share amounts) UNAUDITED  For the quarter  For the year ended December 31,  ended December 31, 2025  2024  2025  2024 Net revenues $ 5,144.5   $ 4,874.0   $ 21,321.9   $ 19,838.2  Cost of goods sold  (3,390.6 )   (3,163.1 )   (13,611.7 )   (12,757.7 ) Selling and administrative expenses  (934.9 )   (903.3 )   (3,742.8 )   (3,580.4 ) Operating income  819.0    807.6    3,967.4    3,500.1  Interest expense  (55.6 )   (59.9 )   (226.7 )   (238.4 ) Other income/(expense), net  (22.1 )   2.8    (62.1 )   (19.9 ) Earnings before income taxes  741.3    750.5    3,678.6    3,241.8  Provision for income taxes  (122.8 )   (135.2 )   (705.9 )   (627.6 ) Earnings from continuing operations  618.5    615.3    2,972.7    2,614.2  Discontinued operations, net of tax  (21.6 )   (3.4 )   (37.0 )   (24.7 ) Net earnings  596.9    611.9    2,935.7    2,589.5  Less: Net earnings from continuing operations attributable to noncontrolling interests  (5.6 )   (7.6 )   (17.1 )   (21.6 ) Net earnings attributable to Trane Technologies plc $ 591.3   $ 604.3   $ 2,918.6   $ 2,567.9          Amounts attributable to Trane Technologies plc ordinary shareholders:        Continuing operations $ 612.9   $ 607.7   $ 2,955.6   $ 2,592.6  Discontinued operations  (21.6 )   (3.4 )   (37.0 )   (24.7 ) Net earnings $ 591.3   $ 604.3   $ 2,918.6   $ 2,567.9          Diluted earnings (loss) per share attributable to Trane Technologies plc ordinary shareholder:        Continuing operations $ 2.74   $ 2.67   $ 13.14   $ 11.35  Discontinued operations  (0.10 )   (0.01 )   (0.16 )   (0.11 ) Net earnings $ 2.64   $ 2.66   $ 12.98   $ 11.24          Weighted-average number of common shares outstanding:        Diluted  223.6    227.3    224.9    228.4  Table 2 TRANE TECHNOLOGIES PLC Reconciliation of GAAP to non-GAAP (In millions, except per share amounts) UNAUDITED   For the quarter ended December 31, 2025  For the year ended December 31, 2025   As    As  As    As   Reported  Adjustments  Adjusted  Reported  Adjustments  Adjusted  Net revenues $ 5,144.5   $ —   $ 5,144.5   $ 21,321.9   $ —   $ 21,321.9                Operating income  819.0    17.7  (a,b)  836.7    3,967.4    (22.8 ) (a,b,c)  3,944.6   Operating margin  15.9 %     16.3 %   18.6 %     18.5 %               Earnings from continuing operations before income taxes  741.3    34.9  (a,b,d)  776.2    3,678.6    (5.6 ) (a,b,c,d)  3,673.0   Provision for income taxes  (122.8 )   (8.8 ) (e)  (131.6 )   (705.9 )   (13.9 ) (e)  (719.8 )  Effective tax rate  16.6 %     17.0 %   19.2 %     19.6 %  Earnings from continuing operations attributable to Trane Technologies plc $ 612.9   $ 26.1  (f) $ 639.0   $ 2,955.6   $ (19.5 ) (f) $ 2,936.1                Diluted earnings per common share             Continuing operations $ 2.74   $ 0.12   $ 2.86   $ 13.14   $ (0.08 )  $ 13.06                Weighted-average number of common shares outstanding:             Diluted  223.6    —    223.6    224.9    —    224.9                Detail of Adjustments:            (a) Restructuring costs (COGS &amp; SG&amp;A)   $ 13.6       $ 31.2    (b) M&amp;A transaction costs (SG&amp;A)    4.1        7.2    (c) Non-cash adjustments for contingent consideration (SG&amp;A)    —        (61.2 )   (d) Non-cash settlement charge related to the transfer of a pension liability to an insurance company    17.2        17.2    (e) Tax impact of adjustments (a,b,d)    (8.8 )       (13.9 )   (f) Impact of adjustments on earnings from continuing operations attributable to Trane Technologies plc   $ 26.1       $ (19.5 )                 Pre-tax impact of adjustments on cost of goods sold   $ 3.0       $ 7.5     Pre-tax impact of adjustments on selling &amp; administrative expenses    14.7        (30.3 )    Pre-tax impact of adjustments on operating income   $ 17.7       $ (22.8 )    Pre-tax impact of adjustments on other, net    17.2        17.2     Pre-tax impact of adjustments on earnings from continuing operations   $ 34.9       $ (5.6 )   Table 3 TRANE TECHNOLOGIES PLC Reconciliation of GAAP to non-GAAP (In millions, except per share amounts) UNAUDITED   For the quarter ended December 31, 2024  For the year ended December 31, 2024   As    As  As    As   Reported  Adjustments  Adjusted  Reported  Adjustments  Adjusted  Net revenues $ 4,874.0   $ —   $ 4,874.0   $ 19,838.2   $ —   $ 19,838.2                Operating income  807.6    (13.2 ) (a,b,c,d)  794.4    3,500.1    (13.3 ) (a,b,c,d)  3,486.8   Operating margin  16.6 %     16.3 %   17.6 %     17.6 %               Earnings from continuing operations before income taxes  750.5    (13.2 ) (a,b,c,d)  737.3    3,241.8    (13.3 ) (a,b,c,d)  3,228.5   Provision for income taxes  (135.2 )   (1.6 ) (f)  (136.8 )   (627.6 )   (16.8 ) (e,f)  (644.4 )  Effective tax rate  18.0 %     18.6 %   19.4 %     20.0 %  Earnings from continuing operations attributable to Trane Technologies plc $ 607.7   $ (14.8 ) (g) $ 592.9   $ 2,592.6   $ (30.1 ) (g) $ 2,562.5                Diluted earnings per common share             Continuing operations $ 2.67   $ (0.06 )  $ 2.61   $ 11.35   $ (0.13 )  $ 11.22                Weighted-average number of common shares outstanding:             Diluted  227.3    —    227.3    228.4    —    228.4                Detail of Adjustments:            (a) Restructuring costs (COGS &amp; SG&amp;A)   $ 1.5       $ 5.1    (b) Legacy legal liability (SG&amp;A)    (1.1 )       2.4    (c) M&amp;A transaction costs (SG&amp;A)    2.5        4.2    (d) Non-cash adjustments for contingent consideration (SG&amp;A)    (16.1 )       (25.0 )   (e) U.S. discrete tax benefit    —        (12.9 )   (f) Tax impact of adjustments (a,b,c)    (1.6 )       (3.9 )   (g) Impact of adjustments on earnings from continuing operations attributable to Trane Technologies plc   $ (14.8 )      $ (30.1 )                 Pre-tax impact of adjustments on cost of goods sold   $ 0.1       $ (1.0 )    Pre-tax impact of adjustments on selling &amp; administrative expenses    (13.3 )       (12.3 )    Pre-tax impact of adjustments on operating income   $ (13.2 )      $ (13.3 )   Table 4 TRANE TECHNOLOGIES PLC Reconciliation of GAAP to non-GAAP (In millions) UNAUDITED   For the quarter ended December 31, 2025  For the quarter ended December 31, 2024   As Reported  Margin  As Reported  Margin Americas Net revenues $ 4,012.6     $ 3,802.5              Segment operating income $ 686.7   17.1 %  $ 685.0   18.0 %  Restructuring/Other(a)  5.1   0.1 %   (15.7 )  (0.4 )%  Adjusted operating income *  691.8   17.2 %   669.3   17.6 %  Depreciation and amortization  70.1   1.8 %   76.0   2.0 %  Other income/(expense), net(c)  (4.7 )  (0.1 )%   (3.9 )  (0.1 )%  Adjusted EBITDA * $ 757.2   18.9 %  $ 741.4   19.5 %          EMEA Net revenues $ 771.0     $ 690.3              Segment operating income $ 122.0   15.8 %  $ 119.8   17.4 %  Restructuring/Other(a)  2.6   0.4 %   (0.7 )  (0.1 )%  Adjusted operating income *  124.6   16.2 %   119.1   17.3 %  Depreciation and amortization  11.2   1.4 %   11.1   1.6 %  Other income/(expense), net  (2.1 )  (0.3 )%   0.2   — %  Adjusted EBITDA * $ 133.7   17.3 %  $ 130.4   18.9 %          Asia Pacific Net revenues $ 360.9     $ 381.2              Segment operating income $ 92.7   25.7 %  $ 94.3   24.7 %  Restructuring/Other(a)  —   — %   1.8   0.5 %  Adjusted operating income *  92.7   25.7 %   96.1   25.2 %  Depreciation and amortization  3.6   1.0 %   4.6   1.2 %  Other income/(expense), net  (1.3 )  (0.4 )%   0.2   0.1 %  Adjusted EBITDA * $ 95.0   26.3 %  $ 100.9   26.5 %          Corporate Unallocated corporate expense $ (82.4 )    $ (91.5 )    Restructuring/Other(b)  10.0      1.4     Adjusted corporate expense *  (72.4 )     (90.1 )    Depreciation and amortization  5.9      5.1     Other income/(expense), net(c)  3.2      6.3     Adjusted EBITDA * $ (63.3 )    $ (78.7 )            Total Company Net revenues $ 5,144.5     $ 4,874.0              Operating income $ 819.0   15.9 %  $ 807.6   16.6 %  Restructuring/Other(a,b)  17.7   0.4 %   (13.2 )  (0.3 )%  Adjusted operating income  836.7   16.3 %   794.4   16.3 %  Depreciation and amortization  90.8   1.7 %   96.8   2.0 %  Other income/(expense), net(c)  (4.9 )  (0.1 )%   2.8   — %  Adjusted EBITDA * $ 922.6   17.9 %  $ 894.0   18.3 % *Represents a non-GAAP measure, refer to pages 6-7 in the Earnings Release for definitions. (a) Restructuring/Other in 2025 and 2024 includes restructuring amounts unless specified otherwise. Restructuring/Other within Americas in 2024 includes $16.1 million non-cash adjustment for contingent consideration. (b) Restructuring/Other within Corporate in 2025 includes $4.1M of M&amp;A transaction costs. Restructuring/Other within Corporate in 2024 includes $1.1M of legacy legal liability and $2.5M of M&amp;A transaction costs. (c) Other income/(expense), net in 2025 has been adjusted to exclude $17.2M non-cash settlement charge related to the transfer of a pension liability to an insurance company, with $5.0M in Americas and $12.2M in Corporate. Table 5 TRANE TECHNOLOGIES PLC Reconciliation of GAAP to non-GAAP (In millions) UNAUDITED   For the year ended December 31, 2025  For the year ended December 31, 2024   As Reported  Margin  As Reported  Margin Americas Net revenues $ 17,168.8     $ 15,903.2              Segment operating income $ 3,479.4   20.3 %  $ 3,061.8   19.3 %  Restructuring/Other(a)  (40.4 )  (0.3 )%   (22.7 )  (0.2 )%  Adjusted operating income *  3,439.0   20.0 %   3,039.1   19.1 %  Depreciation and amortization  294.5   1.7 %   299.8   1.9 %  Other income/(expense), net(c)  (20.1 )  (0.1 )%   (20.6 )  (0.1 )%  Adjusted EBITDA * $ 3,713.4   21.6 %  $ 3,318.3   20.9 %          EMEA Net revenues $ 2,802.1     $ 2,556.7              Segment operating income $ 475.1   17.0 %  $ 472.4   18.5 %  Restructuring/Other(a)  3.5   0.1 %   0.4   — %  Adjusted operating income *  478.6   17.1 %   472.8   18.5 %  Depreciation and amortization  44.2   1.6 %   43.5   1.7 %  Other income/(expense), net  (10.1 )  (0.4 )%   (11.2 )  (0.4 )%  Adjusted EBITDA * $ 512.7   18.3 %  $ 505.1   19.8 %          Asia Pacific Net revenues $ 1,351.0     $ 1,378.3              Segment operating income $ 307.1   22.7 %  $ 307.0   22.3 %  Restructuring/Other(a)  1.0   0.1 %   1.8   0.1 %  Adjusted operating income *  308.1   22.8 %   308.8   22.4 %  Depreciation and amortization  15.8   1.2 %   17.9   1.3 %  Other income/(expense), net  (0.4 )  (0.1 )%   2.6   0.2 %  Adjusted EBITDA * $ 323.5   23.9 %  $ 329.3   23.9 %          Corporate Unallocated corporate expense $ (294.2 )    $ (341.1 )    Restructuring/Other(b)  13.1      7.2     Adjusted corporate expense *  (281.1 )     (333.9 )    Depreciation and amortization  21.8      18.2     Other income/(expense), net(c)  (14.3 )     9.3     Adjusted EBITDA * $ (273.6 )    $ (306.4 )            Total Company Net revenues $ 21,321.9     $ 19,838.2              Operating income $ 3,967.4   18.6 %  $ 3,500.1   17.6 %  Restructuring/Other (a,b)  (22.8 )  (0.1 )%   (13.3 )  — %  Adjusted operating income  3,944.6   18.5 %   3,486.8   17.6 %  Depreciation and amortization  376.3   1.8 %   379.4   1.9 %  Other income/(expense), net(c)  (44.9 )  (0.2 )%   (19.9 )  (0.1 )%  Adjusted EBITDA * $ 4,276.0   20.1 %  $ 3,846.3   19.4 % *Represents a non-GAAP measure, refer to pages 6-7 in the Earnings Release for definitions. (a) Restructuring/Other in 2025 and 2024 includes restructuring amounts unless specified otherwise. Restructuring/Other within Americas in 2025 includes $61.2M non cash adjustment for contingent consideration. Restructuring/Other within Americas in 2024 includes $25.0M non cash adjustment for contingent consideration. (b) Restructuring/Other within Corporate in 2025 includes $7.2M of M&amp;A transaction costs. Restructuring/Other within Corporate in 2024 includes $2.4M of legacy legal liability and $4.2M of M&amp;A transaction costs. (c) Other income/(expense), net in 2025 has been adjusted to exclude $17.2M non-cash settlement charge related to the transfer of a pension liability to an insurance company, with $5.0M in Americas and $12.2M in Corporate. Table 6 TRANE TECHNOLOGIES PLC Reconciliation of GAAP to non-GAAP (In millions) UNAUDITED  For the quarter  ended December 31,  2025  2024 Total Company    Adjusted EBITDA * $ 922.6   $ 894.0  Less: items to reconcile adjusted EBITDA to net earnings attributable to Trane Technologies plc    Depreciation and amortization  (90.8 )   (96.8 ) Interest expense  (55.6 )   (59.9 ) Provision for income taxes  (122.8 )   (135.2 ) Restructuring costs  (13.6 )   (1.5 ) M&amp;A transaction costs  (4.1 )   (2.5 ) Non-cash adjustments for contingent consideration  —    16.1  Non-cash settlement charge related to the transfer of a pension liability to an insurance company  (17.2 )   —  Legacy legal liability  —    1.1  Discontinued operations, net of tax  (21.6 )   (3.4 ) Net earnings from continuing operations attributable to noncontrolling interests  (5.6 )   (7.6 ) Net earnings attributable to Trane Technologies plc $ 591.3   $ 604.3  *Represents a non-GAAP measure, refer to pages 6-7 in the Earnings Release for definitions. Table 7 TRANE TECHNOLOGIES PLC Reconciliation of GAAP to non-GAAP (In millions) UNAUDITED  For the year  ended December 31,  2025  2024 Total Company    Adjusted EBITDA * $ 4,276.0   $ 3,846.3  Less: items to reconcile adjusted EBITDA to net earnings attributable to Trane Technologies plc    Depreciation and amortization  (376.3 )   (379.4 ) Interest expense  (226.7 )   (238.4 ) Provision for income taxes  (705.9 )   (627.6 ) Restructuring costs  (31.2 )   (5.1 ) M&amp;A transaction costs  (7.2 )   (4.2 ) Non-cash adjustments for contingent consideration  61.2    25.0  Non-cash settlement charge related to the transfer of a pension liability to an insurance company  (17.2 )   —  Legacy legal liability  —    (2.4 ) Discontinued operations, net of tax  (37.0 )   (24.7 ) Net earnings from continuing operations attributable to noncontrolling interests  (17.1 )   (21.6 ) Net earnings attributable to Trane Technologies plc $ 2,918.6   $ 2,567.9  *Represents a non-GAAP measure, refer to pages 6-7 in the Earnings Release for definitions. Table 8 TRANE TECHNOLOGIES PLC Condensed Consolidated Balance Sheets (In millions) UNAUDITED  December 31,  December 31,  2025  2024 ASSETS    Cash and cash equivalents $ 1,763.3  $ 1,590.1 Accounts and notes receivable, net  3,235.3    3,090.2  Inventories  2,103.6    1,971.5  Other current assets  760.8    686.0  Total current assets  7,863.0    7,337.8  Property, plant and equipment, net  2,251.3    2,024.5  Goodwill  6,457.0    6,127.9  Intangible assets, net  3,236.7    3,308.2  Other noncurrent assets  1,612.7    1,348.3  Total assets $ 21,420.7   $ 20,146.7      LIABILITIES AND EQUITY    Accounts payable $ 2,153.9   $ 2,148.0  Accrued expenses and other current liabilities  3,439.8    3,468.7  Short-term borrowings and current maturities of long-term debt  693.0    452.2  Total current liabilities  6,286.7    6,068.9  Long-term debt  3,922.1    4,318.1  Other noncurrent liabilities  2,611.0    2,272.8  Total equity  8,600.9    7,486.9  Total liabilities and equity $ 21,420.7   $ 20,146.7  Table 9 TRANE TECHNOLOGIES PLC Condensed Consolidated Statement of Cash Flows (In millions) UNAUDITED  For the year  ended December 31,  2025  2024 Operating Activities    Earnings from continuing operations $ 2,972.7   $ 2,614.2  Depreciation and amortization  376.3    379.4  Changes in assets and liabilities and other non-cash items  (128.6 )   184.1  Net cash provided by (used in) continuing operating activities  3,220.4    3,177.7  Net cash provided by (used in) discontinued operating activities  (25.9 )   (32.1 ) Net cash provided by (used in) operating activities  3,194.5    3,145.6      Investing Activities    Capital expenditures, net  (383.0 )   (370.6 ) Acquisition of businesses, net of cash acquired  (276.0 )   (180.3 ) Other investing activities, net  19.0    (12.0 ) Net cash provided by (used in) investing activities  (640.0 )   (562.9 )     Financing Activities    Net proceeds from (payments of) debt  (159.1 )   (9.0 ) Dividends paid to ordinary shareholders  (837.3 )   (757.5 ) Repurchase of ordinary shares  (1,481.3 )   (1,280.8 ) Other financing activities, net  (18.1 )   26.7  Net cash provided by (used in) financing activities  (2,495.8 )   (2,020.6 )     Effect of exchange rate changes on cash and cash equivalents  114.5    (67.3 ) Net increase (decrease) in cash and cash equivalents  173.2    494.8  Cash and cash equivalents - beginning of period  1,590.1    1,095.3  Cash and cash equivalents - end of period $ 1,763.3   $ 1,590.1  Table 10 TRANE TECHNOLOGIES PLC Balance Sheet Metrics and Free Cash Flow ($ in millions) UNAUDITED   December 31,  December 31,    2025    2024  Net Receivables  $ 3,235.3   $ 3,090.2  Days Sales Outstanding   57.4    57.9       Net Inventory  $ 2,103.6   $ 1,971.5  Inventory Turns   6.4    6.4       Accounts Payable  $ 2,153.9   $ 2,148.0  Days Payable Outstanding   58.0    62.0  --------------------------------------------------------------------------------------------</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>https://investors.tranetechnologies.com/news-and-events/news-releases/news-release-details/2026/Trane-Technologies-Reports-Strong-Fourth-Quarter-and-Full-Year-2025-Results-Robust-Bookings-and-Backlog-Provide-Strong-Visibility-Entering-2026/default.aspx</t>
-        </is>
-      </c>
+          <t>SWORDS, Ireland--(BUSINESS WIRE)-- 
+Trane Technologies plc (NYSE:TT), a global climate innovator, announced the Board of Directors has approved a 12% increase to the company’s dividend, resulting in a quarterly dividend of $1.05 per ordinary share, or $4.20 per share annualized. The dividend is payable March 31, 2026, to shareholders of record on March 6, 2026. “Our purpose-driven strategy, disciplined execution and relentless investment in growth and innovation enables us to consistently deliver a leading growth profile, strong margins and powerful free cash flow,” said Dave Regnery, chair and CEO, Trane Technologies. “Since launching Trane Technologies in 2020, we have delivered free cash flow conversion of 106% of adjusted net earnings, enabling us to execute our balanced capital allocation strategy and nearly double the dividend. We are well positioned to deliver continued strong financial performance and differentiated shareholder returns over the long term.” Today’s announcement reflects the Company’s confidence in its ability to generate strong free cash flow in the future and pay a competitive and growing dividend over time. The Company has paid consecutive quarterly cash dividends on its common shares since 1919 and annual dividends since 1910.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>Trane Technologies</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>https://investors.tranetechnologies.com/news-and-events/news-releases/news-release-details/2026/Trane-Technologies-Increases-Dividend-by-12-Declares-Quarterly-Dividend/default.aspx</t>
         </is>
       </c>
     </row>

</xml_diff>